<commit_message>
found a bug where BWMP scores in the input data were incorrect
</commit_message>
<xml_diff>
--- a/Outputs/10_lepa_per_metric_comparison.xlsx
+++ b/Outputs/10_lepa_per_metric_comparison.xlsx
@@ -613,70 +613,70 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LTR127_2015</t>
+          <t>LTR386_2019</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LTR127</t>
+          <t>LTR386</t>
         </is>
       </c>
       <c r="C4">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="D4">
-        <v>0.1666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F4">
-        <v>0.1666666666666667</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>0.3888888888888889</v>
+        <v>0.746031746031746</v>
       </c>
       <c r="H4">
-        <v>0.3888888888888888</v>
+        <v>0.746031746031746</v>
       </c>
       <c r="I4">
-        <v>1.110223024625157E-16</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>0.06666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="K4">
-        <v>0.06666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>0.6198132780082988</v>
+        <v>0.7766089108910891</v>
       </c>
       <c r="N4">
-        <v>0.4680962343096234</v>
+        <v>0.5198019801980198</v>
       </c>
       <c r="O4">
-        <v>0.1517170436986754</v>
+        <v>0.2568069306930693</v>
       </c>
       <c r="P4">
-        <v>0.31</v>
+        <v>0.66</v>
       </c>
       <c r="Q4">
-        <v>0.23</v>
+        <v>0.59</v>
       </c>
       <c r="R4">
-        <v>0.07999999999999999</v>
+        <v>0.07000000000000006</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Bad</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U4" t="b">
@@ -686,61 +686,61 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LTR386_2019</t>
+          <t>LTR163_2022</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LTR386</t>
+          <t>LTR163</t>
         </is>
       </c>
       <c r="C5">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D5">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E5">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>0.746031746031746</v>
+        <v>0.7564102564102564</v>
       </c>
       <c r="H5">
-        <v>0.746031746031746</v>
+        <v>0.7654320987654321</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>-0.009021842355175669</v>
       </c>
       <c r="J5">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K5">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>0.7766089108910891</v>
+        <v>0.7742011278195489</v>
       </c>
       <c r="N5">
-        <v>0.5198019801980198</v>
+        <v>0.5106132075471698</v>
       </c>
       <c r="O5">
-        <v>0.2568069306930693</v>
+        <v>0.2635879202723791</v>
       </c>
       <c r="P5">
-        <v>0.66</v>
+        <v>0.79</v>
       </c>
       <c r="Q5">
-        <v>0.59</v>
+        <v>0.73</v>
       </c>
       <c r="R5">
-        <v>0.07000000000000006</v>
+        <v>0.06000000000000005</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -749,90 +749,90 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LTR163_2022</t>
+          <t>LTR127_2015</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LTR163</t>
+          <t>LTR127</t>
         </is>
       </c>
       <c r="C6">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="D6">
-        <v>0.8333333333333334</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E6">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="G6">
-        <v>0.7564102564102564</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="H6">
-        <v>0.7654320987654321</v>
+        <v>0.4523809523809523</v>
       </c>
       <c r="I6">
-        <v>-0.009021842355175669</v>
+        <v>-0.06349206349206338</v>
       </c>
       <c r="J6">
-        <v>0.8</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="K6">
-        <v>0.8</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>0.7742011278195489</v>
+        <v>0.6198132780082988</v>
       </c>
       <c r="N6">
-        <v>0.5106132075471698</v>
+        <v>0.4680962343096234</v>
       </c>
       <c r="O6">
-        <v>0.2635879202723791</v>
+        <v>0.1517170436986754</v>
       </c>
       <c r="P6">
-        <v>0.79</v>
+        <v>0.31</v>
       </c>
       <c r="Q6">
-        <v>0.73</v>
+        <v>0.25</v>
       </c>
       <c r="R6">
-        <v>0.06000000000000005</v>
+        <v>0.06</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Bad</t>
         </is>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LTR127_2017</t>
+          <t>LTR127_2020</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -841,25 +841,25 @@
         </is>
       </c>
       <c r="C7">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="D7">
-        <v>0.1666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="E7">
-        <v>0.1666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="F7">
-        <v>-5.551115123125783E-17</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>0.4333333333333333</v>
+        <v>0.5777777777777778</v>
       </c>
       <c r="H7">
-        <v>0.3888888888888888</v>
+        <v>0.6041666666666666</v>
       </c>
       <c r="I7">
-        <v>0.04444444444444456</v>
+        <v>-0.0263888888888888</v>
       </c>
       <c r="J7">
         <v>0.2</v>
@@ -871,31 +871,31 @@
         <v>0</v>
       </c>
       <c r="M7">
-        <v>0.640194489465154</v>
+        <v>0.62902706185567</v>
       </c>
       <c r="N7">
-        <v>0.4558346839546191</v>
+        <v>0.390222293814433</v>
       </c>
       <c r="O7">
-        <v>0.1843598055105349</v>
+        <v>0.238804768041237</v>
       </c>
       <c r="P7">
-        <v>0.36</v>
+        <v>0.48</v>
       </c>
       <c r="Q7">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="R7">
         <v>0.06</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U7" t="b">
@@ -905,70 +905,70 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LTR127_2020</t>
+          <t>LTR450_2015</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LTR127</t>
+          <t>LTR450</t>
         </is>
       </c>
       <c r="C8">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="D8">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E8">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>0.5777777777777778</v>
+        <v>0.5277777777777778</v>
       </c>
       <c r="H8">
-        <v>0.5888888888888889</v>
+        <v>0.5277777777777778</v>
       </c>
       <c r="I8">
-        <v>-0.01111111111111107</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>0.2</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="K8">
-        <v>0.2</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>0.62902706185567</v>
+        <v>0.6028761061946902</v>
       </c>
       <c r="N8">
-        <v>0.390222293814433</v>
+        <v>0.3429203539823009</v>
       </c>
       <c r="O8">
-        <v>0.238804768041237</v>
+        <v>0.2599557522123893</v>
       </c>
       <c r="P8">
-        <v>0.48</v>
+        <v>0.38</v>
       </c>
       <c r="Q8">
-        <v>0.42</v>
+        <v>0.32</v>
       </c>
       <c r="R8">
         <v>0.06</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="U8" t="b">
@@ -978,147 +978,147 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LTR450_2015</t>
+          <t>LTR1466_2019</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LTR450</t>
+          <t>LTR1466</t>
         </is>
       </c>
       <c r="C9">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="D9">
-        <v>0.3333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E9">
-        <v>0.3333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0.5277777777777778</v>
+        <v>0.7283950617283951</v>
       </c>
       <c r="H9">
-        <v>0.5277777777777778</v>
+        <v>0.7202380952380952</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>0.008156966490299844</v>
       </c>
       <c r="J9">
-        <v>0.06666666666666667</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>0.06666666666666667</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>0.06666666666666665</v>
       </c>
       <c r="M9">
-        <v>0.6028761061946902</v>
+        <v>0.7776280323450135</v>
       </c>
       <c r="N9">
-        <v>0.3429203539823009</v>
+        <v>0.6024258760107817</v>
       </c>
       <c r="O9">
-        <v>0.2599557522123893</v>
+        <v>0.1752021563342319</v>
       </c>
       <c r="P9">
-        <v>0.38</v>
+        <v>0.83</v>
       </c>
       <c r="Q9">
-        <v>0.32</v>
+        <v>0.77</v>
       </c>
       <c r="R9">
-        <v>0.06</v>
+        <v>0.05999999999999994</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LTR1466_2019</t>
+          <t>LTR127_2017</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LTR1466</t>
+          <t>LTR127</t>
         </is>
       </c>
       <c r="C10">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="D10">
-        <v>0.8333333333333334</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E10">
-        <v>0.8333333333333334</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>-5.551115123125783E-17</v>
       </c>
       <c r="G10">
-        <v>0.7283950617283951</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="H10">
-        <v>0.7202380952380952</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="I10">
-        <v>0.008156966490299844</v>
+        <v>5.551115123125783E-17</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="K10">
-        <v>0.9333333333333333</v>
+        <v>0.2</v>
       </c>
       <c r="L10">
-        <v>0.06666666666666665</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>0.7776280323450135</v>
+        <v>0.640194489465154</v>
       </c>
       <c r="N10">
-        <v>0.6024258760107817</v>
+        <v>0.4558346839546191</v>
       </c>
       <c r="O10">
-        <v>0.1752021563342319</v>
+        <v>0.1843598055105349</v>
       </c>
       <c r="P10">
-        <v>0.83</v>
+        <v>0.36</v>
       </c>
       <c r="Q10">
-        <v>0.77</v>
+        <v>0.31</v>
       </c>
       <c r="R10">
-        <v>0.05999999999999994</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="U10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1367,10 +1367,10 @@
         <v>0.782051282051282</v>
       </c>
       <c r="H14">
-        <v>0.7884615384615384</v>
+        <v>0.7901234567901233</v>
       </c>
       <c r="I14">
-        <v>-0.006410256410256387</v>
+        <v>-0.008072174738841253</v>
       </c>
       <c r="J14">
         <v>0.4666666666666667</v>
@@ -2024,10 +2024,10 @@
         <v>0.7799999999999999</v>
       </c>
       <c r="H23">
-        <v>0.7799999999999999</v>
+        <v>0.7820512820512823</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>-0.002051282051282355</v>
       </c>
       <c r="J23">
         <v>0.6</v>
@@ -2657,70 +2657,70 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LTR1063_2021</t>
+          <t>LTR86_2016</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LTR1063</t>
+          <t>LTR86</t>
         </is>
       </c>
       <c r="C32">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="D32">
-        <v>0.1666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E32">
-        <v>0.1666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="F32">
-        <v>-5.551115123125783E-17</v>
+        <v>-0.1666666666666667</v>
       </c>
       <c r="G32">
-        <v>0.3958333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H32">
-        <v>0.3958333333333333</v>
+        <v>0.6893939393939394</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>-0.02272727272727282</v>
       </c>
       <c r="J32">
-        <v>0.2</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="K32">
-        <v>0.2</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="L32">
-        <v>0</v>
+        <v>2.775557561562891E-17</v>
       </c>
       <c r="M32">
-        <v>0.6405693950177935</v>
+        <v>0.7788944723618091</v>
       </c>
       <c r="N32">
-        <v>0.567170818505338</v>
+        <v>0.6752512562814069</v>
       </c>
       <c r="O32">
-        <v>0.07339857651245552</v>
+        <v>0.1036432160804022</v>
       </c>
       <c r="P32">
-        <v>0.35</v>
+        <v>0.48</v>
       </c>
       <c r="Q32">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="R32">
-        <v>0.01999999999999996</v>
+        <v>-0.02000000000000002</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U32" t="b">
@@ -2730,58 +2730,58 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LTR308_2018</t>
+          <t>LTR1063_2021</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LTR308</t>
+          <t>LTR1063</t>
         </is>
       </c>
       <c r="C33">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="D33">
-        <v>0.3333333333333333</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E33">
-        <v>0.3333333333333333</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>-5.551115123125783E-17</v>
       </c>
       <c r="G33">
-        <v>0.3541666666666667</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="H33">
-        <v>0.3541666666666667</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="I33">
         <v>0</v>
       </c>
       <c r="J33">
-        <v>0.1333333333333333</v>
+        <v>0.2</v>
       </c>
       <c r="K33">
-        <v>0.1333333333333333</v>
+        <v>0.2</v>
       </c>
       <c r="L33">
-        <v>2.775557561562891E-17</v>
+        <v>0</v>
       </c>
       <c r="M33">
-        <v>0.6134259259259259</v>
+        <v>0.6405693950177935</v>
       </c>
       <c r="N33">
-        <v>0.5324074074074073</v>
+        <v>0.567170818505338</v>
       </c>
       <c r="O33">
-        <v>0.0810185185185186</v>
+        <v>0.07339857651245552</v>
       </c>
       <c r="P33">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="Q33">
-        <v>0.34</v>
+        <v>0.33</v>
       </c>
       <c r="R33">
         <v>0.01999999999999996</v>
@@ -2803,70 +2803,70 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LTR1447_2022</t>
+          <t>LTR308_2018</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>LTR1447</t>
+          <t>LTR308</t>
         </is>
       </c>
       <c r="C34">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="D34">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E34">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
-        <v>0.7828282828282829</v>
+        <v>0.3541666666666667</v>
       </c>
       <c r="H34">
-        <v>0.7828282828282829</v>
+        <v>0.3541666666666667</v>
       </c>
       <c r="I34">
         <v>0</v>
       </c>
       <c r="J34">
-        <v>0.6</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="K34">
-        <v>0.6</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="L34">
-        <v>0</v>
+        <v>2.775557561562891E-17</v>
       </c>
       <c r="M34">
-        <v>1.052013422818792</v>
+        <v>0.6134259259259259</v>
       </c>
       <c r="N34">
-        <v>1.042506720430108</v>
+        <v>0.5324074074074073</v>
       </c>
       <c r="O34">
-        <v>0.009506702388683896</v>
+        <v>0.0810185185185186</v>
       </c>
       <c r="P34">
-        <v>0.78</v>
+        <v>0.36</v>
       </c>
       <c r="Q34">
-        <v>0.77</v>
+        <v>0.34</v>
       </c>
       <c r="R34">
-        <v>0.01000000000000001</v>
+        <v>0.01999999999999996</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="U34" t="b">
@@ -2876,70 +2876,70 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LTR1488_2019</t>
+          <t>LTR1447_2022</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LTR1488</t>
+          <t>LTR1447</t>
         </is>
       </c>
       <c r="C35">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D35">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E35">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>0.6666666666666666</v>
+        <v>0.7828282828282829</v>
       </c>
       <c r="H35">
-        <v>0.6960784313725491</v>
+        <v>0.7843137254901961</v>
       </c>
       <c r="I35">
-        <v>-0.02941176470588247</v>
+        <v>-0.001485442661913194</v>
       </c>
       <c r="J35">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="K35">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="L35">
         <v>0</v>
       </c>
       <c r="M35">
-        <v>0.6811097256857854</v>
+        <v>1.052013422818792</v>
       </c>
       <c r="N35">
-        <v>0.6795511221945136</v>
+        <v>1.042506720430108</v>
       </c>
       <c r="O35">
-        <v>0.001558603491271793</v>
+        <v>0.009506702388683896</v>
       </c>
       <c r="P35">
-        <v>0.51</v>
+        <v>0.78</v>
       </c>
       <c r="Q35">
-        <v>0.52</v>
+        <v>0.77</v>
       </c>
       <c r="R35">
-        <v>-0.01000000000000001</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U35" t="b">
@@ -2949,70 +2949,70 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LTR1488_2022</t>
+          <t>LTR1449_2015</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>LTR1488</t>
+          <t>LTR1449</t>
         </is>
       </c>
       <c r="C36">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="D36">
-        <v>0.3333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E36">
-        <v>0.3333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>0.5800000000000001</v>
+        <v>0.7698412698412698</v>
       </c>
       <c r="H36">
-        <v>0.576923076923077</v>
+        <v>0.7999999999999999</v>
       </c>
       <c r="I36">
-        <v>0.003076923076923088</v>
+        <v>-0.03015873015873016</v>
       </c>
       <c r="J36">
-        <v>0.1333333333333333</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="K36">
-        <v>0.1333333333333333</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="L36">
-        <v>2.775557561562891E-17</v>
+        <v>0</v>
       </c>
       <c r="M36">
-        <v>0.625</v>
+        <v>0.6937919463087248</v>
       </c>
       <c r="N36">
-        <v>0.5909653465346534</v>
+        <v>0.6937919463087248</v>
       </c>
       <c r="O36">
-        <v>0.03403465346534662</v>
+        <v>0</v>
       </c>
       <c r="P36">
-        <v>0.42</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q36">
-        <v>0.41</v>
+        <v>0.7</v>
       </c>
       <c r="R36">
-        <v>0.01000000000000001</v>
+        <v>-0.01000000000000001</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U36" t="b">
@@ -3022,34 +3022,34 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LTR1492_2016</t>
+          <t>LTR1488_2019</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LTR1492</t>
+          <t>LTR1488</t>
         </is>
       </c>
       <c r="C37">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="D37">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="E37">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="F37">
         <v>0</v>
       </c>
       <c r="G37">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H37">
-        <v>0.6111111111111112</v>
+        <v>0.7037037037037037</v>
       </c>
       <c r="I37">
-        <v>-0.01111111111111118</v>
+        <v>-0.03703703703703709</v>
       </c>
       <c r="J37">
         <v>0.2</v>
@@ -3061,22 +3061,22 @@
         <v>0</v>
       </c>
       <c r="M37">
-        <v>0.6772113022113021</v>
+        <v>0.6811097256857854</v>
       </c>
       <c r="N37">
-        <v>0.6342137592137592</v>
+        <v>0.6795511221945136</v>
       </c>
       <c r="O37">
-        <v>0.04299754299754288</v>
+        <v>0.001558603491271793</v>
       </c>
       <c r="P37">
-        <v>0.45</v>
+        <v>0.51</v>
       </c>
       <c r="Q37">
-        <v>0.44</v>
+        <v>0.52</v>
       </c>
       <c r="R37">
-        <v>0.01000000000000001</v>
+        <v>-0.01000000000000001</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -3095,34 +3095,34 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LTR1501_2016</t>
+          <t>LTR1488_2022</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LTR1501</t>
+          <t>LTR1488</t>
         </is>
       </c>
       <c r="C38">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="D38">
         <v>0.3333333333333333</v>
       </c>
       <c r="E38">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F38">
-        <v>-0.1666666666666667</v>
+        <v>0</v>
       </c>
       <c r="G38">
-        <v>0.753968253968254</v>
+        <v>0.5800000000000001</v>
       </c>
       <c r="H38">
-        <v>0.753968253968254</v>
+        <v>0.5864197530864197</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>-0.006419753086419622</v>
       </c>
       <c r="J38">
         <v>0.1333333333333333</v>
@@ -3134,19 +3134,19 @@
         <v>2.775557561562891E-17</v>
       </c>
       <c r="M38">
-        <v>0.6205568720379147</v>
+        <v>0.625</v>
       </c>
       <c r="N38">
-        <v>0.4102488151658767</v>
+        <v>0.5909653465346534</v>
       </c>
       <c r="O38">
-        <v>0.210308056872038</v>
+        <v>0.03403465346534662</v>
       </c>
       <c r="P38">
-        <v>0.46</v>
+        <v>0.42</v>
       </c>
       <c r="Q38">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="R38">
         <v>0.01000000000000001</v>
@@ -3168,58 +3168,58 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LTR1687_2017</t>
+          <t>LTR1492_2016</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LTR1687</t>
+          <t>LTR1492</t>
         </is>
       </c>
       <c r="C39">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="D39">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E39">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>0.576923076923077</v>
+        <v>0.6</v>
       </c>
       <c r="H39">
-        <v>0.576923076923077</v>
+        <v>0.6111111111111112</v>
       </c>
       <c r="I39">
-        <v>0</v>
+        <v>-0.01111111111111118</v>
       </c>
       <c r="J39">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="K39">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L39">
         <v>0</v>
       </c>
       <c r="M39">
-        <v>0.6631679389312978</v>
+        <v>0.6772113022113021</v>
       </c>
       <c r="N39">
-        <v>0.625</v>
+        <v>0.6342137592137592</v>
       </c>
       <c r="O39">
-        <v>0.03816793893129777</v>
+        <v>0.04299754299754288</v>
       </c>
       <c r="P39">
-        <v>0.54</v>
+        <v>0.45</v>
       </c>
       <c r="Q39">
-        <v>0.53</v>
+        <v>0.44</v>
       </c>
       <c r="R39">
         <v>0.01000000000000001</v>
@@ -3241,31 +3241,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LTR297_2015</t>
+          <t>LTR1501_2016</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>LTR297</t>
+          <t>LTR1501</t>
         </is>
       </c>
       <c r="C40">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="D40">
         <v>0.3333333333333333</v>
       </c>
       <c r="E40">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>-0.1666666666666667</v>
       </c>
       <c r="G40">
-        <v>0.4166666666666667</v>
+        <v>0.753968253968254</v>
       </c>
       <c r="H40">
-        <v>0.4166666666666667</v>
+        <v>0.753968253968254</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -3280,31 +3280,31 @@
         <v>2.775557561562891E-17</v>
       </c>
       <c r="M40">
-        <v>0.5686475409836065</v>
+        <v>0.6205568720379147</v>
       </c>
       <c r="N40">
-        <v>0.5122950819672131</v>
+        <v>0.4102488151658767</v>
       </c>
       <c r="O40">
-        <v>0.05635245901639341</v>
+        <v>0.210308056872038</v>
       </c>
       <c r="P40">
-        <v>0.36</v>
+        <v>0.46</v>
       </c>
       <c r="Q40">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="R40">
         <v>0.01000000000000001</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U40" t="b">
@@ -3314,70 +3314,70 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LTR337_2016</t>
+          <t>LTR1687_2017</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>LTR337</t>
+          <t>LTR1687</t>
         </is>
       </c>
       <c r="C41">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="D41">
-        <v>0.8333333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="E41">
-        <v>0.8333333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="F41">
         <v>0</v>
       </c>
       <c r="G41">
-        <v>0.7388888888888889</v>
+        <v>0.576923076923077</v>
       </c>
       <c r="H41">
-        <v>0.7388888888888889</v>
+        <v>0.576923076923077</v>
       </c>
       <c r="I41">
         <v>0</v>
       </c>
       <c r="J41">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="K41">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="L41">
         <v>0</v>
       </c>
       <c r="M41">
-        <v>0.7444707740916271</v>
+        <v>0.6631679389312978</v>
       </c>
       <c r="N41">
-        <v>0.7192930489731437</v>
+        <v>0.625</v>
       </c>
       <c r="O41">
-        <v>0.02517772511848337</v>
+        <v>0.03816793893129777</v>
       </c>
       <c r="P41">
-        <v>0.78</v>
+        <v>0.54</v>
       </c>
       <c r="Q41">
-        <v>0.77</v>
+        <v>0.53</v>
       </c>
       <c r="R41">
         <v>0.01000000000000001</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U41" t="b">
@@ -3387,70 +3387,70 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LTR337_2022</t>
+          <t>LTR297_2015</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LTR337</t>
+          <t>LTR297</t>
         </is>
       </c>
       <c r="C42">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="D42">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E42">
-        <v>0.8333333333333334</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F42">
-        <v>-0.1666666666666667</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>0.7222222222222222</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H42">
-        <v>0.7156862745098039</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="I42">
-        <v>0.006535947712418277</v>
+        <v>0</v>
       </c>
       <c r="J42">
-        <v>0.8</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="K42">
-        <v>0.8</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="L42">
-        <v>0</v>
+        <v>2.775557561562891E-17</v>
       </c>
       <c r="M42">
-        <v>0.759308510638298</v>
+        <v>0.5686475409836065</v>
       </c>
       <c r="N42">
-        <v>0.6490384615384616</v>
+        <v>0.5122950819672131</v>
       </c>
       <c r="O42">
-        <v>0.1102700490998364</v>
+        <v>0.05635245901639341</v>
       </c>
       <c r="P42">
-        <v>0.74</v>
+        <v>0.36</v>
       </c>
       <c r="Q42">
-        <v>0.75</v>
+        <v>0.35</v>
       </c>
       <c r="R42">
-        <v>-0.01000000000000001</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="U42" t="b">
@@ -3460,70 +3460,70 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LTR351_2019</t>
+          <t>LTR337_2016</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LTR351</t>
+          <t>LTR337</t>
         </is>
       </c>
       <c r="C43">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="D43">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E43">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F43">
         <v>0</v>
       </c>
       <c r="G43">
-        <v>0.7045454545454546</v>
+        <v>0.7388888888888889</v>
       </c>
       <c r="H43">
-        <v>0.7045454545454547</v>
+        <v>0.7388888888888889</v>
       </c>
       <c r="I43">
-        <v>-1.110223024625157E-16</v>
+        <v>0</v>
       </c>
       <c r="J43">
-        <v>0.2666666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="K43">
-        <v>0.2666666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="L43">
-        <v>-5.551115123125783E-17</v>
+        <v>0</v>
       </c>
       <c r="M43">
-        <v>0.6763059701492536</v>
+        <v>0.7444707740916271</v>
       </c>
       <c r="N43">
-        <v>0.6669776119402985</v>
+        <v>0.7192930489731437</v>
       </c>
       <c r="O43">
-        <v>0.009328358208955168</v>
+        <v>0.02517772511848337</v>
       </c>
       <c r="P43">
-        <v>0.54</v>
+        <v>0.78</v>
       </c>
       <c r="Q43">
-        <v>0.53</v>
+        <v>0.77</v>
       </c>
       <c r="R43">
         <v>0.01000000000000001</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U43" t="b">
@@ -3533,12 +3533,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LTR411_2022</t>
+          <t>LTR337_2022</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LTR411</t>
+          <t>LTR337</t>
         </is>
       </c>
       <c r="C44">
@@ -3548,46 +3548,46 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="E44">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>-0.1666666666666667</v>
       </c>
       <c r="G44">
-        <v>0.8076923076923076</v>
+        <v>0.7222222222222222</v>
       </c>
       <c r="H44">
-        <v>0.8266666666666667</v>
+        <v>0.7156862745098039</v>
       </c>
       <c r="I44">
-        <v>-0.01897435897435906</v>
+        <v>0.006535947712418277</v>
       </c>
       <c r="J44">
-        <v>0.7333333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="K44">
-        <v>0.7333333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="L44">
         <v>0</v>
       </c>
       <c r="M44">
-        <v>0.7774122807017543</v>
+        <v>0.759308510638298</v>
       </c>
       <c r="N44">
-        <v>0.7214912280701754</v>
+        <v>0.6490384615384616</v>
       </c>
       <c r="O44">
-        <v>0.05592105263157887</v>
+        <v>0.1102700490998364</v>
       </c>
       <c r="P44">
+        <v>0.74</v>
+      </c>
+      <c r="Q44">
         <v>0.75</v>
       </c>
-      <c r="Q44">
-        <v>0.74</v>
-      </c>
       <c r="R44">
-        <v>0.01000000000000001</v>
+        <v>-0.01000000000000001</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
@@ -3606,61 +3606,61 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LTR86_2016</t>
+          <t>LTR351_2019</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LTR86</t>
+          <t>LTR351</t>
         </is>
       </c>
       <c r="C45">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="D45">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="E45">
         <v>0.5</v>
       </c>
       <c r="F45">
-        <v>-0.1666666666666667</v>
+        <v>0</v>
       </c>
       <c r="G45">
-        <v>0.6666666666666666</v>
+        <v>0.7045454545454546</v>
       </c>
       <c r="H45">
-        <v>0.6666666666666666</v>
+        <v>0.7045454545454547</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>-1.110223024625157E-16</v>
       </c>
       <c r="J45">
-        <v>0.1333333333333333</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="K45">
-        <v>0.1333333333333333</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="L45">
-        <v>2.775557561562891E-17</v>
+        <v>-5.551115123125783E-17</v>
       </c>
       <c r="M45">
-        <v>0.7788944723618091</v>
+        <v>0.6763059701492536</v>
       </c>
       <c r="N45">
-        <v>0.6752512562814069</v>
+        <v>0.6669776119402985</v>
       </c>
       <c r="O45">
-        <v>0.1036432160804022</v>
+        <v>0.009328358208955168</v>
       </c>
       <c r="P45">
-        <v>0.48</v>
+        <v>0.54</v>
       </c>
       <c r="Q45">
-        <v>0.49</v>
+        <v>0.53</v>
       </c>
       <c r="R45">
-        <v>-0.01000000000000001</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LTR1502_2019</t>
+          <t>LTR411_2022</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LTR1502</t>
+          <t>LTR411</t>
         </is>
       </c>
       <c r="C46">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D46">
         <v>0.6666666666666666</v>
@@ -3700,49 +3700,49 @@
         <v>0</v>
       </c>
       <c r="G46">
-        <v>0.6666666666666666</v>
+        <v>0.8076923076923076</v>
       </c>
       <c r="H46">
-        <v>0.6666666666666666</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="I46">
-        <v>0</v>
+        <v>-0.03846153846153855</v>
       </c>
       <c r="J46">
-        <v>0.2666666666666667</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="K46">
-        <v>0.2666666666666667</v>
+        <v>0.7333333333333333</v>
       </c>
       <c r="L46">
-        <v>-5.551115123125783E-17</v>
+        <v>0</v>
       </c>
       <c r="M46">
-        <v>0.6867283950617283</v>
+        <v>0.7774122807017543</v>
       </c>
       <c r="N46">
-        <v>0.6327160493827161</v>
+        <v>0.7214912280701754</v>
       </c>
       <c r="O46">
-        <v>0.05401234567901225</v>
+        <v>0.05592105263157887</v>
       </c>
       <c r="P46">
-        <v>0.57</v>
+        <v>0.75</v>
       </c>
       <c r="Q46">
-        <v>0.5600000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="R46">
-        <v>0.009999999999999898</v>
+        <v>0.01000000000000001</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U46" t="b">
@@ -3752,12 +3752,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LTR337_2019</t>
+          <t>LTR1502_2019</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LTR337</t>
+          <t>LTR1502</t>
         </is>
       </c>
       <c r="C47">
@@ -3773,10 +3773,10 @@
         <v>0</v>
       </c>
       <c r="G47">
-        <v>0.6590909090909091</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H47">
-        <v>0.6590909090909091</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -3791,13 +3791,13 @@
         <v>-5.551115123125783E-17</v>
       </c>
       <c r="M47">
-        <v>0.6812339331619538</v>
+        <v>0.6867283950617283</v>
       </c>
       <c r="N47">
-        <v>0.6411082474226804</v>
+        <v>0.6327160493827161</v>
       </c>
       <c r="O47">
-        <v>0.04012568573927344</v>
+        <v>0.05401234567901225</v>
       </c>
       <c r="P47">
         <v>0.57</v>
@@ -3825,70 +3825,70 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LTR1063_2017</t>
+          <t>LTR337_2019</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LTR1063</t>
+          <t>LTR337</t>
         </is>
       </c>
       <c r="C48">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="D48">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E48">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F48">
         <v>0</v>
       </c>
       <c r="G48">
-        <v>0.4166666666666667</v>
+        <v>0.6590909090909091</v>
       </c>
       <c r="H48">
-        <v>0.4166666666666667</v>
+        <v>0.6590909090909091</v>
       </c>
       <c r="I48">
         <v>0</v>
       </c>
       <c r="J48">
-        <v>0.06666666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="K48">
-        <v>0.06666666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="L48">
-        <v>0</v>
+        <v>-5.551115123125783E-17</v>
       </c>
       <c r="M48">
-        <v>0.6305661577608143</v>
+        <v>0.6812339331619538</v>
       </c>
       <c r="N48">
-        <v>0.6242048346055979</v>
+        <v>0.6411082474226804</v>
       </c>
       <c r="O48">
-        <v>0.006361323155216314</v>
+        <v>0.04012568573927344</v>
       </c>
       <c r="P48">
-        <v>0.36</v>
+        <v>0.57</v>
       </c>
       <c r="Q48">
-        <v>0.36</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="R48">
-        <v>0</v>
+        <v>0.009999999999999898</v>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U48" t="b">
@@ -3898,70 +3898,70 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LTR1299_2015</t>
+          <t>LTR1063_2017</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LTR1299</t>
+          <t>LTR1063</t>
         </is>
       </c>
       <c r="C49">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F49">
         <v>0</v>
       </c>
       <c r="G49">
-        <v>0.9782608695652174</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H49">
-        <v>0.9855072463768115</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="I49">
-        <v>-0.007246376811594124</v>
+        <v>0</v>
       </c>
       <c r="J49">
-        <v>0.9333333333333333</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="K49">
-        <v>0.9333333333333333</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="L49">
         <v>0</v>
       </c>
       <c r="M49">
-        <v>0.79053480475382</v>
+        <v>0.6305661577608143</v>
       </c>
       <c r="N49">
-        <v>0.79053480475382</v>
+        <v>0.6242048346055979</v>
       </c>
       <c r="O49">
-        <v>0</v>
+        <v>0.006361323155216314</v>
       </c>
       <c r="P49">
-        <v>0.93</v>
+        <v>0.36</v>
       </c>
       <c r="Q49">
-        <v>0.93</v>
+        <v>0.36</v>
       </c>
       <c r="R49">
         <v>0</v>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="U49" t="b">
@@ -3971,7 +3971,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LTR1299_2019</t>
+          <t>LTR1299_2015</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3980,49 +3980,49 @@
         </is>
       </c>
       <c r="C50">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="D50">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="E50">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="F50">
         <v>0</v>
       </c>
       <c r="G50">
-        <v>0.9242424242424243</v>
+        <v>0.9782608695652174</v>
       </c>
       <c r="H50">
-        <v>0.9318181818181818</v>
+        <v>1.007246376811594</v>
       </c>
       <c r="I50">
-        <v>-0.007575757575757458</v>
+        <v>-0.02898550724637661</v>
       </c>
       <c r="J50">
-        <v>0.8</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="K50">
-        <v>0.8</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="L50">
         <v>0</v>
       </c>
       <c r="M50">
-        <v>0.7226138828633406</v>
+        <v>0.79053480475382</v>
       </c>
       <c r="N50">
-        <v>0.7226138828633405</v>
+        <v>0.79053480475382</v>
       </c>
       <c r="O50">
-        <v>1.110223024625157E-16</v>
+        <v>0</v>
       </c>
       <c r="P50">
-        <v>0.82</v>
+        <v>0.93</v>
       </c>
       <c r="Q50">
-        <v>0.82</v>
+        <v>0.93</v>
       </c>
       <c r="R50">
         <v>0</v>
@@ -4044,7 +4044,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LTR1299_2022</t>
+          <t>LTR1299_2019</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4053,49 +4053,49 @@
         </is>
       </c>
       <c r="C51">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F51">
         <v>0</v>
       </c>
       <c r="G51">
-        <v>0.9074074074074074</v>
+        <v>0.9242424242424243</v>
       </c>
       <c r="H51">
-        <v>0.9120370370370371</v>
+        <v>0.9318181818181818</v>
       </c>
       <c r="I51">
-        <v>-0.00462962962962965</v>
+        <v>-0.007575757575757458</v>
       </c>
       <c r="J51">
-        <v>1.266666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="K51">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="L51">
-        <v>0.06666666666666665</v>
+        <v>0</v>
       </c>
       <c r="M51">
-        <v>0.9577287946428572</v>
+        <v>0.7226138828633406</v>
       </c>
       <c r="N51">
-        <v>0.9556361607142857</v>
+        <v>0.7226138828633405</v>
       </c>
       <c r="O51">
-        <v>0.002092633928571508</v>
+        <v>1.110223024625157E-16</v>
       </c>
       <c r="P51">
-        <v>1</v>
+        <v>0.82</v>
       </c>
       <c r="Q51">
-        <v>1</v>
+        <v>0.82</v>
       </c>
       <c r="R51">
         <v>0</v>
@@ -4117,16 +4117,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LTR1320_2016</t>
+          <t>LTR1299_2022</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LTR1320</t>
+          <t>LTR1299</t>
         </is>
       </c>
       <c r="C52">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -4138,31 +4138,31 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>0.9464285714285715</v>
+        <v>0.9074074074074074</v>
       </c>
       <c r="H52">
-        <v>0.9464285714285715</v>
+        <v>0.9259259259259259</v>
       </c>
       <c r="I52">
-        <v>0</v>
+        <v>-0.01851851851851849</v>
       </c>
       <c r="J52">
-        <v>1.533333333333333</v>
+        <v>1.266666666666667</v>
       </c>
       <c r="K52">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="L52">
-        <v>0.1333333333333335</v>
+        <v>0.06666666666666665</v>
       </c>
       <c r="M52">
-        <v>0.8657495256166983</v>
+        <v>0.9577287946428572</v>
       </c>
       <c r="N52">
-        <v>0.8657495256166983</v>
+        <v>0.9556361607142857</v>
       </c>
       <c r="O52">
-        <v>0</v>
+        <v>0.002092633928571508</v>
       </c>
       <c r="P52">
         <v>1</v>
@@ -4190,7 +4190,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LTR1320_2019</t>
+          <t>LTR1320_2016</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4199,61 +4199,61 @@
         </is>
       </c>
       <c r="C53">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="D53">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="E53">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
       <c r="G53">
-        <v>0.8571428571428572</v>
+        <v>0.9464285714285715</v>
       </c>
       <c r="H53">
-        <v>0.8571428571428572</v>
+        <v>0.9642857142857143</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>-0.01785714285714279</v>
       </c>
       <c r="J53">
-        <v>0.6666666666666666</v>
+        <v>1.533333333333333</v>
       </c>
       <c r="K53">
-        <v>0.6666666666666666</v>
+        <v>1.4</v>
       </c>
       <c r="L53">
-        <v>0</v>
+        <v>0.1333333333333335</v>
       </c>
       <c r="M53">
-        <v>0.6916199158485272</v>
+        <v>0.8657495256166983</v>
       </c>
       <c r="N53">
-        <v>0.6916199158485273</v>
+        <v>0.8657495256166983</v>
       </c>
       <c r="O53">
-        <v>-1.110223024625157E-16</v>
+        <v>0</v>
       </c>
       <c r="P53">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="Q53">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="R53">
         <v>0</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="U53" t="b">
@@ -4263,7 +4263,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LTR1320_2022</t>
+          <t>LTR1320_2019</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4272,61 +4272,61 @@
         </is>
       </c>
       <c r="C54">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>0.9482758620689654</v>
+        <v>0.8571428571428572</v>
       </c>
       <c r="H54">
-        <v>0.9482758620689654</v>
+        <v>0.8560606060606061</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>0.001082251082251129</v>
       </c>
       <c r="J54">
-        <v>1.066666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="K54">
-        <v>1.066666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="L54">
-        <v>-4.440892098500626E-16</v>
+        <v>0</v>
       </c>
       <c r="M54">
-        <v>0.9419642857142857</v>
+        <v>0.6916199158485272</v>
       </c>
       <c r="N54">
-        <v>0.9433285509325681</v>
+        <v>0.6916199158485273</v>
       </c>
       <c r="O54">
-        <v>-0.001364265218282368</v>
+        <v>-1.110223024625157E-16</v>
       </c>
       <c r="P54">
-        <v>0.99</v>
+        <v>0.76</v>
       </c>
       <c r="Q54">
-        <v>0.99</v>
+        <v>0.76</v>
       </c>
       <c r="R54">
         <v>0</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U54" t="b">
@@ -4336,16 +4336,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LTR1379_2015</t>
+          <t>LTR1320_2022</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LTR1379</t>
+          <t>LTR1320</t>
         </is>
       </c>
       <c r="C55">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -4357,37 +4357,37 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>0.9545454545454546</v>
+        <v>0.9482758620689654</v>
       </c>
       <c r="H55">
-        <v>0.9545454545454547</v>
+        <v>0.9655172413793104</v>
       </c>
       <c r="I55">
-        <v>-1.110223024625157E-16</v>
+        <v>-0.01724137931034497</v>
       </c>
       <c r="J55">
-        <v>0.9333333333333333</v>
+        <v>1.066666666666667</v>
       </c>
       <c r="K55">
-        <v>0.9333333333333333</v>
+        <v>1.066666666666667</v>
       </c>
       <c r="L55">
-        <v>0</v>
+        <v>-4.440892098500626E-16</v>
       </c>
       <c r="M55">
-        <v>0.782323883161512</v>
+        <v>0.9419642857142857</v>
       </c>
       <c r="N55">
-        <v>0.781786941580756</v>
+        <v>0.9433285509325681</v>
       </c>
       <c r="O55">
-        <v>0.0005369415807560118</v>
+        <v>-0.001364265218282368</v>
       </c>
       <c r="P55">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="Q55">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="R55">
         <v>0</v>
@@ -4409,7 +4409,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LTR1379_2019</t>
+          <t>LTR1379_2015</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4418,61 +4418,61 @@
         </is>
       </c>
       <c r="C56">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="D56">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="E56">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="F56">
         <v>0</v>
       </c>
       <c r="G56">
-        <v>0.8623188405797101</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="H56">
-        <v>0.8623188405797101</v>
+        <v>0.9696969696969697</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>-0.01515151515151514</v>
       </c>
       <c r="J56">
-        <v>0.6</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="K56">
-        <v>0.6</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="L56">
         <v>0</v>
       </c>
       <c r="M56">
-        <v>0.7549055232558139</v>
+        <v>0.782323883161512</v>
       </c>
       <c r="N56">
-        <v>0.7549055232558139</v>
+        <v>0.781786941580756</v>
       </c>
       <c r="O56">
-        <v>0</v>
+        <v>0.0005369415807560118</v>
       </c>
       <c r="P56">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="Q56">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="R56">
         <v>0</v>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="U56" t="b">
@@ -4482,7 +4482,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LTR1379_2022</t>
+          <t>LTR1379_2019</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4491,49 +4491,49 @@
         </is>
       </c>
       <c r="C57">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D57">
-        <v>0.8333333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E57">
-        <v>0.8333333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F57">
         <v>0</v>
       </c>
       <c r="G57">
-        <v>0.8064516129032259</v>
+        <v>0.8623188405797101</v>
       </c>
       <c r="H57">
-        <v>0.8064516129032259</v>
+        <v>0.8623188405797101</v>
       </c>
       <c r="I57">
         <v>0</v>
       </c>
       <c r="J57">
-        <v>0.8666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="K57">
-        <v>0.8666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="L57">
         <v>0</v>
       </c>
       <c r="M57">
-        <v>0.6558675699300699</v>
+        <v>0.7549055232558139</v>
       </c>
       <c r="N57">
-        <v>0.6456043956043956</v>
+        <v>0.7549055232558139</v>
       </c>
       <c r="O57">
-        <v>0.01026317432567425</v>
+        <v>0</v>
       </c>
       <c r="P57">
-        <v>0.79</v>
+        <v>0.72</v>
       </c>
       <c r="Q57">
-        <v>0.79</v>
+        <v>0.72</v>
       </c>
       <c r="R57">
         <v>0</v>
@@ -4555,16 +4555,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LTR1385_2016</t>
+          <t>LTR1379_2022</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>LTR1385</t>
+          <t>LTR1379</t>
         </is>
       </c>
       <c r="C58">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="D58">
         <v>0.8333333333333334</v>
@@ -4576,49 +4576,49 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>0.9722222222222222</v>
+        <v>0.8064516129032259</v>
       </c>
       <c r="H58">
-        <v>0.9722222222222222</v>
+        <v>0.8064516129032259</v>
       </c>
       <c r="I58">
         <v>0</v>
       </c>
       <c r="J58">
-        <v>0.6</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="K58">
-        <v>0.6</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="L58">
         <v>0</v>
       </c>
       <c r="M58">
-        <v>0.8421814671814671</v>
+        <v>0.6558675699300699</v>
       </c>
       <c r="N58">
-        <v>0.8421814671814671</v>
+        <v>0.6456043956043956</v>
       </c>
       <c r="O58">
-        <v>0</v>
+        <v>0.01026317432567425</v>
       </c>
       <c r="P58">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="Q58">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="R58">
         <v>0</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U58" t="b">
@@ -4628,7 +4628,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LTR1385_2019</t>
+          <t>LTR1385_2016</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4637,61 +4637,61 @@
         </is>
       </c>
       <c r="C59">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="D59">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E59">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F59">
         <v>0</v>
       </c>
       <c r="G59">
-        <v>0.6833333333333332</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="H59">
-        <v>0.6833333333333332</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="I59">
         <v>0</v>
       </c>
       <c r="J59">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K59">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L59">
         <v>0</v>
       </c>
       <c r="M59">
-        <v>0.7584212662337662</v>
+        <v>0.8421814671814671</v>
       </c>
       <c r="N59">
-        <v>0.7584212662337662</v>
+        <v>0.8421814671814671</v>
       </c>
       <c r="O59">
         <v>0</v>
       </c>
       <c r="P59">
-        <v>0.73</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Q59">
-        <v>0.73</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="R59">
         <v>0</v>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>High</t>
         </is>
       </c>
       <c r="U59" t="b">
@@ -4701,7 +4701,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LTR1385_2022</t>
+          <t>LTR1385_2019</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="C60">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="D60">
         <v>0.6666666666666666</v>
@@ -4722,37 +4722,37 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <v>0.8174603174603176</v>
+        <v>0.6833333333333332</v>
       </c>
       <c r="H60">
-        <v>0.8174603174603176</v>
+        <v>0.6833333333333332</v>
       </c>
       <c r="I60">
         <v>0</v>
       </c>
       <c r="J60">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K60">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="L60">
         <v>0</v>
       </c>
       <c r="M60">
-        <v>0.9122670807453416</v>
+        <v>0.7584212662337662</v>
       </c>
       <c r="N60">
-        <v>0.9130094043887146</v>
+        <v>0.7584212662337662</v>
       </c>
       <c r="O60">
-        <v>-0.0007423236433730107</v>
+        <v>0</v>
       </c>
       <c r="P60">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="Q60">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
       <c r="R60">
         <v>0</v>
@@ -4774,70 +4774,70 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LTR1447_2019</t>
+          <t>LTR1385_2022</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>LTR1447</t>
+          <t>LTR1385</t>
         </is>
       </c>
       <c r="C61">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D61">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E61">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
       <c r="G61">
-        <v>0.7361111111111112</v>
+        <v>0.8174603174603176</v>
       </c>
       <c r="H61">
-        <v>0.7361111111111112</v>
+        <v>0.8174603174603176</v>
       </c>
       <c r="I61">
         <v>0</v>
       </c>
       <c r="J61">
-        <v>0.2666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="K61">
-        <v>0.2666666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="L61">
-        <v>-5.551115123125783E-17</v>
+        <v>0</v>
       </c>
       <c r="M61">
-        <v>0.7019519519519519</v>
+        <v>0.9122670807453416</v>
       </c>
       <c r="N61">
-        <v>0.7019519519519519</v>
+        <v>0.9130094043887146</v>
       </c>
       <c r="O61">
-        <v>0</v>
+        <v>-0.0007423236433730107</v>
       </c>
       <c r="P61">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="Q61">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="R61">
         <v>0</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="U61" t="b">
@@ -4847,70 +4847,70 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LTR1449_2015</t>
+          <t>LTR1447_2019</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LTR1449</t>
+          <t>LTR1447</t>
         </is>
       </c>
       <c r="C62">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="D62">
-        <v>0.8333333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="E62">
-        <v>0.8333333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="F62">
         <v>0</v>
       </c>
       <c r="G62">
-        <v>0.7698412698412698</v>
+        <v>0.7361111111111112</v>
       </c>
       <c r="H62">
-        <v>0.775</v>
+        <v>0.7361111111111112</v>
       </c>
       <c r="I62">
-        <v>-0.005158730158730251</v>
+        <v>0</v>
       </c>
       <c r="J62">
-        <v>0.4666666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="K62">
-        <v>0.4666666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="L62">
-        <v>0</v>
+        <v>-5.551115123125783E-17</v>
       </c>
       <c r="M62">
-        <v>0.6937919463087248</v>
+        <v>0.7019519519519519</v>
       </c>
       <c r="N62">
-        <v>0.6937919463087248</v>
+        <v>0.7019519519519519</v>
       </c>
       <c r="O62">
         <v>0</v>
       </c>
       <c r="P62">
-        <v>0.6899999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="Q62">
-        <v>0.6899999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="R62">
         <v>0</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="U62" t="b">
@@ -4944,10 +4944,10 @@
         <v>0.8409090909090909</v>
       </c>
       <c r="H63">
-        <v>0.8484848484848485</v>
+        <v>0.8478260869565218</v>
       </c>
       <c r="I63">
-        <v>-0.007575757575757569</v>
+        <v>-0.006916996047430901</v>
       </c>
       <c r="J63">
         <v>0.3333333333333333</v>
@@ -5236,10 +5236,10 @@
         <v>0.7901234567901234</v>
       </c>
       <c r="H67">
-        <v>0.7901234567901233</v>
+        <v>0.808641975308642</v>
       </c>
       <c r="I67">
-        <v>1.110223024625157E-16</v>
+        <v>-0.0185185185185186</v>
       </c>
       <c r="J67">
         <v>0.4666666666666667</v>
@@ -5382,10 +5382,10 @@
         <v>0.9019607843137255</v>
       </c>
       <c r="H69">
-        <v>0.9019607843137255</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="I69">
-        <v>0</v>
+        <v>-0.01470588235294112</v>
       </c>
       <c r="J69">
         <v>0.6666666666666666</v>
@@ -5674,10 +5674,10 @@
         <v>0.7011494252873564</v>
       </c>
       <c r="H73">
-        <v>0.7011494252873564</v>
+        <v>0.7055555555555556</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>-0.004406130268199249</v>
       </c>
       <c r="J73">
         <v>0.4</v>
@@ -5820,10 +5820,10 @@
         <v>0.7701149425287356</v>
       </c>
       <c r="H75">
-        <v>0.7758620689655172</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="I75">
-        <v>-0.005747126436781658</v>
+        <v>-0.00766283524904221</v>
       </c>
       <c r="J75">
         <v>0.2</v>
@@ -5893,10 +5893,10 @@
         <v>0.8253968253968255</v>
       </c>
       <c r="H76">
-        <v>0.8253968253968256</v>
+        <v>0.8257575757575757</v>
       </c>
       <c r="I76">
-        <v>-1.110223024625157E-16</v>
+        <v>-0.0003607503607502283</v>
       </c>
       <c r="J76">
         <v>0.6666666666666666</v>
@@ -6540,22 +6540,22 @@
         <v>82</v>
       </c>
       <c r="C3">
-        <v>0.001072238521249652</v>
+        <v>-0.003034997622772077</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0.005026380955348395</v>
+        <v>0.008000955722806301</v>
       </c>
       <c r="F3">
-        <v>0.9964892565883873</v>
+        <v>0.9948954977090645</v>
       </c>
       <c r="G3">
-        <v>5.986467335472058E-88</v>
+        <v>1.845644815360817E-81</v>
       </c>
       <c r="H3">
-        <v>68.29268292682927</v>
+        <v>58.53658536585365</v>
       </c>
     </row>
     <row r="4">
@@ -6624,22 +6624,22 @@
         <v>82</v>
       </c>
       <c r="C6">
-        <v>0.01463414634146341</v>
+        <v>0.01402439024390243</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0.01780487804878049</v>
+        <v>0.01768292682926829</v>
       </c>
       <c r="F6">
-        <v>0.9908736580695875</v>
+        <v>0.9911315006021287</v>
       </c>
       <c r="G6">
-        <v>2.120992596125486E-71</v>
+        <v>6.773526914327024E-72</v>
       </c>
       <c r="H6">
-        <v>43.90243902439025</v>
+        <v>42.68292682926829</v>
       </c>
     </row>
   </sheetData>
@@ -6799,7 +6799,7 @@
         <v>82</v>
       </c>
       <c r="D5">
-        <v>0.699</v>
+        <v>0.703</v>
       </c>
       <c r="E5">
         <v>0.171</v>
@@ -6811,7 +6811,7 @@
         <v>0.25</v>
       </c>
       <c r="H5">
-        <v>0.986</v>
+        <v>1.007</v>
       </c>
     </row>
     <row r="6">
@@ -6982,7 +6982,7 @@
         <v>0.591</v>
       </c>
       <c r="E11">
-        <v>0.19</v>
+        <v>0.189</v>
       </c>
       <c r="F11">
         <v>0.59</v>
@@ -7076,19 +7076,19 @@
         <v>82</v>
       </c>
       <c r="C3">
-        <v>0.0011</v>
+        <v>-0.003</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="F3">
-        <v>0.996</v>
+        <v>0.995</v>
       </c>
       <c r="G3">
-        <v>68.3</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="4">
@@ -7151,19 +7151,19 @@
         <v>82</v>
       </c>
       <c r="C6">
-        <v>0.0146</v>
+        <v>0.014</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0.0178</v>
+        <v>0.0177</v>
       </c>
       <c r="F6">
         <v>0.991</v>
       </c>
       <c r="G6">
-        <v>43.9</v>
+        <v>42.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>